<commit_message>
feat(10-01): generate complete expert review XLSX with 60 questions
Two sets of 30 questions each (beginner/intermediate/advanced),
2 per keyword, across separate tabs for expert reviewer distribution.
</commit_message>
<xml_diff>
--- a/services/benchmarks/results/expert_preview.xlsx
+++ b/services/benchmarks/results/expert_preview.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expert Review" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Set 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Set 2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1884,6 +1885,1326 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DB7D"/>
   <dataValidations count="1">
+    <dataValidation sqref="H2:H31 I2:I31 J2:J31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>question_text</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>correct_answer</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>options</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>explanation</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>source_document</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>difficulty_level</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>factual_correctness</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>pedagogical_alignment</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>source_fidelity</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>rationale</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>According to the excerpt, what types of actions might indicate a child or young person is experiencing emotional or mental health difficulties?</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A) A) Regularly missing whole days at school; B) B) Excelling in all academic subjects; C) C) Actively participating in extracurricular activities; D) D) Consistently arriving early for class</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>The excerpt lists various forms of non-attendance that can suggest underlying emotional or mental health struggles.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>common signs and symptoms</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr"/>
+      <c r="I2" s="4" t="inlineStr"/>
+      <c r="J2" s="4" t="inlineStr"/>
+      <c r="K2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>According to the passage, what is another term used for school absence due to mental wellbeing difficulties?</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A) A) Emotionally Based School Avoidance (EBSA); B) B) Academic Stress; C) C) Physical Illnesses; D) D) Bullying</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The passage provides alternative terms for school absence rooted in mental wellbeing.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>common signs and symptoms</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>According to the excerpt, what can be a cause of reduced school attendance?</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>A) A) Emotional issues; B) B) Physical illnesses; C) C) Lack of transportation; D) D) Family vacations</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>The excerpt states that non-attendance can be rooted in emotional, mental health, or wellbeing issues.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>peer aggression</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>According to preliminary research, which of the following are adults with knowledge of child MHPs more likely to do?</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A) A)  Recognize child MHPs and seek help; B) B) Induce mental health problems in children; C) C) Avoid seeking information about child MHPs; D) D) Disregard the impact of MHPs on children</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>The passage highlights a correlation between knowledge of MHPs and help-seeking behaviors.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>johnson2023_teacher_mh_literacy_review.pdf</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>peer aggression</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>According to the excerpt, which of these is NOT a potential indicator of non-attendance in school?</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>A) A) Prolonged absence from school; B) B) Regularly missing entire days; C) C) Social evaluation fears; D) D) Not attending certain classes</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>The provided excerpt discusses non-attendance reasons related to emotional, mental health, or well-being issues.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>social evaluation fears</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr"/>
+      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>According to the passage, which of the following is NOT a social-emotional skill that can help adolescents succeed in school?</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A) A) Managing goal- and task-directed behavior; B) B) Taking care of their own well-being; C) C) Avoiding social interaction ; D) D) Establishing and maintaining positive social interactions</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The passage lists several skills that help adolescents succeed in school, including managing goal-directed behavior and establishing positive social interactions. </t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>huttunen2025_socioemotional_profiles_anxiety.pdf</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>social evaluation fears</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>According to the excerpt, what type of issue can be related to school attendance?</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A) A) Somatic complaints; B) B) Physical education difficulties; C) C) Extracurricular activity overload; D) D) Technological issues with learning platforms</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>The excerpt states that school attendance problems can be rooted in emotional, mental health, or wellbeing issues.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>somatic complaints</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>According to the text, which of the following is NOT a social-emotional skill that helps adolescents cope with challenges in school?</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>A) A) Managing goal- and task-directed behavior; B) B) Experiencing physical symptoms in response to stress; C) C) Establishing and maintaining positive social interactions; D) D) Achieving academic success</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>The passage lists the skills that help adolescents,  and somatic complaints are not among them.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>huttunen2025_socioemotional_profiles_anxiety.pdf</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>somatic complaints</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>What does the excerpt mention as potential examples of non-attendance?</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>A) A) Attending class but not participating   B) Arriving late to school C) Being absent for entire days or periods D) Completing homework assignments on time</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>The question asks about what the excerpt mentions as potential examples of non-attendance.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>attendance tracking</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>According to the abstract, how do difficulties junior adolescents experience impact their school lives?</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>A) A) They lead to improved academic performance and well-being.; B) B) They cause a decrease in academic performance, behavioral problems, and health deterioration.; C) C) They have no significant impact on school life.; D) D) They result in increased social interaction and extracurricular participation.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>The abstract specifically details the negative consequences junior adolescents face due to academic difficulties.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>shamionov2021_wellbeing_anxiety_variations.pdf</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>attendance tracking</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>According to the excerpt, which is NOT a possible reason for reduced school attendance?</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>A) A) Emotional issues; B) B) Mental health challenges; C) C) Bullying from classmates; D) D) Physical illness</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>The provided excerpt focuses on emotional and mental wellbeing as reasons behind school absence.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>school social climate</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>According to the passage, what is one way that social-emotional skills can help adolescents thrive in school?</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>A) A) Reduce stress related to homework and tests.; B) B) Improve communication with teachers and peers.; C) C) Boost self-confidence for athletic pursuits.; D) D) Increase the likelihood of getting a good night's sleep.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>The passage explains that social-emotional skills benefit students by helping them interact positively with others at school.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>huttunen2025_socioemotional_profiles_anxiety.pdf</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>school social climate</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>According to the excerpt, which type of school absence might be an indicator of underlying emotional or mental health concerns for a child?</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>A) A) Arriving late to class frequently.; B) B) Participating actively in all lessons.; C) C) Leaving early for extracurricular activities.; D) D) Prolonged periods of non-attendance.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Student absences, especially prolonged ones, can be a sign of issues that impact mental wellbeing.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>student–teacher relations</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>According to the excerpt, which of these is NOT a social-emotional skill that can help adolescents thrive in school?</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>A) A) Managing goal- and task-directed behavior; B) B) Establishing and maintaining positive social interactions; C) C) Directly resolving conflicts between students and teachers; D) D) Taking care of their own well-being</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>The excerpt focuses on skills students need to manage themselves and interact positively. Resolving teacher-student conflicts is a separate dynamic.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>huttunen2025_socioemotional_profiles_anxiety.pdf</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>student–teacher relations</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>According to the excerpt, what might cause a child or young person to miss school?</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>A) A) Emotional, mental health, or wellbeing issues; B) B) A lack of interest in their schoolwork; C) C) Financial difficulties within their family; D) D) Bullying from other students</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>The excerpt states that reduced or non-attendance can be rooted in emotional, mental health, or wellbeing issues.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>cognitive restructuring</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>According to the provided text, which of the following strategies might be helpful in addressing 'emotionally based school avoidance'?</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>A) A) Increased physical activity during recess.; B) B) Open communication with parents about homework struggles.; C) C) Engaging in cognitive restructuring techniques to challenge negative thought patterns.; D) D) Implementing stricter consequences for unexcused absences.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>The passage focuses on mental well-being as a root cause of school absence.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>cognitive restructuring</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Which of the following scenarios BEST illustrates an attempt to address the root causes of non-attendance, rather than simply addressing its impacts?</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>A) A) A teacher sends a letter home to parents reminding them about the importance of school attendance.; B) B) Parents and teachers work together to develop a plan to help a student manage their anxiety around attending school.; C) C) The principal calls in students who are frequently absent to discuss the consequences of missing classes.; D) D)  The school counselor keeps track of all absences and reports them to relevant authorities.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Option B focuses on understanding and addressing the underlying emotional or mental health issues that might be causing the student's non-attendance.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>parent-teacher collaboration</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>According to the excerpt, what is a potential benefit of adults having knowledge of child MHPs (mental health problems)?</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>A) A) Increased engagement in parent-teacher collaboration.; B) B) Improved communication with mental health professionals.; C) C) Greater likelihood of seeking out information on managing child MHPs.; D) D) A stronger understanding of the legal ramifications of untreated child MHPs.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>The excerpt highlights the link between knowledge of child MHPs and help-seeking behaviors.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>johnson2023_teacher_mh_literacy_review.pdf</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>parent-teacher collaboration</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Which of the following practices might be considered an example of 'graduated exposure' for a student struggling with school attendance?</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>A) A) Having the student attend only for short periods initially and gradually increase time.; B) B) Requiring parents to send documentation for every missed day.; C) C) Implementing a reward system for perfect attendance throughout the year.; D) D) Suggesting alternative education programs as a full replacement to traditional schooling.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Gradually increasing exposure to school is a common approach in addressing attendance challenges.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>graduated exposure</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>According to the passage, what is the best way to characterize the research findings regarding gender and bullying?</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>A) A) Researchers consistently agree that girls are more likely to be bullied than boys.; B) B) Studies have shown conflicting results about the relationship between gender and bullying.; C) C) Most research suggests that bullying is primarily a problem for young boys.; D) D)  There is limited research available on the topic of gender and bullying.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>The passage states that findings regarding gender in bullying are inconsistent.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>schlesier2023_bullying_anxiety_absenteeism.pdf</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>graduated exposure</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>According to the excerpt, what might be an initial response to mental health or well-being issues that cause non-attendance in school?</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>A) A) Increased parental involvement in the child's education; B) B) Seeking professional counselling for the student; C) C) Implementing stricter attendance policies at school; D) D) Providing extra academic support to help the student catch up</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>This question asks for an initial response, focusing on possible parent actions.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>response systems</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr"/>
+      <c r="I22" s="4" t="inlineStr"/>
+      <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>According to the passage, what system exhibits a strong association with both bullying and anxiety?</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>A) A) Emotional regulation system; B) B) Social interaction system; C) C) Physical response system; D) D) Cognitive appraisal system</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>The passage highlights a connection between bullying, anxiety, and school displeasure.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>schlesier2023_bullying_anxiety_absenteeism.pdf</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>response systems</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>According to the excerpt, what can be a cause of reduced or non-attendance in school?</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>A) A) Emotional issues; B) B) Physical disabilities; C) C) Lack of interest in the curriculum; D) D) Difficulties with homework assignments</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>The excerpt states that non-attendance can stem from emotional, mental health, or wellbeing problems.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>emotion dysregulation</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>According to the passage, which of the following best differentiates social-emotional skills from educational aspirations and school anxiety?</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>A) A) Social-emotional skills are relatively consistent characteristics, while educational aspirations and school anxiety are context-specific experiences.; B) B) Educational aspirations and school anxiety are innate traits, while social-emotional skills are learned behaviors.; C) C) Social-emotional skills primarily influence academic performance, whereas educational aspirations and school anxiety relate to personal well-being.; D) D)  School anxiety is a subset of social-emotional skills, while educational aspirations are independent of them.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>The passage explains that social-emotional skills are consistent traits while educational aspirations and school anxiety arise from the schooling context.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>huttunen2025_socioemotional_profiles_anxiety.pdf</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>emotion dysregulation</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>According to the excerpt, what can be a contributing factor to reduced school attendance?</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>A) A) Physical illness; B) B) Family issues; C) C) Emotional and mental health difficulties; D) D) Lack of academic interest</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>The excerpt states that non-attendance can stem from emotional, mental health, or wellbeing issues.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>comorbid depression</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr"/>
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Which of the following terms does the passage suggest could be used to describe school avoidance linked to mental health?</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>A) A) Comorbid depression; B) B) Emotionally based school avoidance; C) C) Academic burnout; D) D)  Behavioral inhibition</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>The passage lists several terms for school avoidance rooted in mental health.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>comorbid depression</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>According to this passage, which of the following can be a reason for school absenteeism?</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>A) A) Emotional or mental health issues; B) B) Academic difficulties; C) C) Social conflicts with peers; D) D) Lack of interest in extracurricular activities</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>The passage states that reduced attendance can stem from emotional, mental health, or well-being problems.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>internalizing symptoms</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr"/>
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>The passage suggests that research on bullying, school anxiety, and school absenteeism often focuses on these issues as:</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>A) A) Distinct entities that should not be compared.; B) B) Individual problems requiring separate solutions.; C) C) Interconnected constructs that deserve more joint investigation.; D) D) Symptoms of a larger psychological disorder.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>The passage highlights the lack of research combining these factors, implying they are closely related.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>schlesier2023_bullying_anxiety_absenteeism.pdf</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>internalizing symptoms</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr"/>
+      <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>According to the excerpt, what is a possible cause for non-attendance at school?,</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>A) A)  Physical illnesses or health problems.; B) B)  Concerns about academic performance.; C) C)  Difficulties with social interactions.; D) D)  Emotional, mental health, or wellbeing issues.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>The excerpt states that non-attendance is often rooted in emotional or mental health issues.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>autonomic arousal</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr"/>
+      <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>According to the abstract, which of these effects is *indirectly* related to junior adolescents' academic difficulties?</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>A) A) School anxiety; B) B) Academic performance; C) C) Behavioral problems; D) D) Deterioration of health</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Academic difficulties can lead to several consequences, including a decline in overall health.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>shamionov2021_wellbeing_anxiety_variations.pdf</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>autonomic arousal</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DB7D"/>
+  <dataValidations count="1">
     <dataValidation sqref="H2:H31 I2:I31 J2:J31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid rating" error="Please enter a value between 1 and 5" type="list">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
feat: update keyword taxonomy, refine adaptive quiz logic for new users, and update benchmark documentation.
</commit_message>
<xml_diff>
--- a/services/benchmarks/results/expert_preview.xlsx
+++ b/services/benchmarks/results/expert_preview.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Set 1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Set 2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Review" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3211,4 +3212,1318 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>question_text</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>correct_answer</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>options</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>explanation</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>source_document</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>difficulty_level</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>factual_correctness</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>pedagogical_alignment</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>source_fidelity</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>rationale</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>According to the excerpt, which terms are sometimes used alongside 'non-attendance' when discussing mental wellbeing difficulties?</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A) Socially Based School Avoidance (SBSA); B) Emotionally Based School Avoidance (EBSA); C) Academically Based School Non-Attendance; D) Psychologically Driven Education Absence</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>The excerpt states that 'Emotionally Based School Avoidance' is a term sometimes used along with others.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>common signs and symptoms</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="n"/>
+      <c r="I2" s="4" t="n"/>
+      <c r="J2" s="4" t="n"/>
+      <c r="K2" s="4" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>According to the excerpt, what is the primary way CBT helps people manage their feelings or problems?</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A) By suggesting relaxation techniques.; B) By prescribing medication for mental health concerns.; C) By changing thoughts and behaviors.; D) By providing a supportive listening ear.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The excerpt states that CBT helps people by changing the way they think and behave.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>annafreud_seven_ways_support_worried.pdf</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>common signs and symptoms</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="n"/>
+      <c r="K3" s="4" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>According to preliminary research, what effect does knowledge of child MHPs have on helpseeking behaviors?</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>A) It has no effect on helpseeking behaviors.; B) Adults who recognize child MHPs are less likely to seek out professional help.; C) Adults who lack knowledge of child MHPs are more likely to endorse inappropriate professionals as sources of help.; D) Adults with sufficient knowledge of child MHPs for problem recognition are more likely to endorse appropriate professionals and seek help.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>The excerpt states the link between knowledge, recognition, and help-seeking behaviors.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>johnson2023_teacher_mh_literacy_review.pdf</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>peer aggression</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Which of the following is NOT a specific topic mentioned in relation to adolescent mental health in the UK context according to this excerpt?</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A) Increasing rates of self-harm; B) Prevalence of emotional distress among CYP; C) Diagnosable disorders among adolescents; D) Rates of peer aggression among teenagers</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>The provided excerpt does not mention rates of peer aggression.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>troy2022_school_structural_mh_promotion_review.pdf</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>peer aggression</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>According to the excerpt, which of the following is NOT a social-emotional skill that helps adolescents cope with school challenges?</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>A) Managing goal- and task-directed behavior; B) Establishing and maintaining positive social interactions; C) Overcoming social evaluation fears; D) Taking care of their own wellbeing</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>The excerpt lists skills like managing behavior and social interactions, not fears.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>huttunen2025_socioemotional_profiles_anxiety.pdf</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>social evaluation fears</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>According to the passage, what is one way that schools help pupils?</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A) Reduce social evaluation fears; B) Facilitate creative writing; C) Provide access to extracurricular activities; D) Encourage physical education</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>The passage states schools help pupils by developing protective factors.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>social evaluation fears</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="4" t="n"/>
+      <c r="K7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Which of the following is NOT mentioned as a benefit of social-emotional skills for adolescents?</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A) Managing goal- and task-directed behavior; B) Establishing and maintaining positive social interactions; C) Taking care of their own wellbeing; D) Experiencing reduced somatic complaints</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>The excerpt focuses on positive aspects of social-emotional skills like academic success and well-being.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>huttunen2025_socioemotional_profiles_anxiety.pdf</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>somatic complaints</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>According to the passage, what is the primary function of schools?</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>A) To provide meals for students; B) To address somatic complaints in pupils; C) To develop protective factors in their pupils; D) To establish strict behavioral rules</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>The passage states that schools play a crucial role in developing protective factors.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>somatic complaints</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="n"/>
+      <c r="J9" s="4" t="n"/>
+      <c r="K9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>What is NOT mentioned as a potential outcome of school anxiety and poor academic wellbeing in junior adolescents?</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>A) Deterioration of health; B) Improved attendance; C) Behavioral problems; D) Decrease in academic performance</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>The excerpt describes negative outcomes associated with school anxiety and poor well-being.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>shamionov2021_wellbeing_anxiety_variations.pdf</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>attendance tracking</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>According to the abstract, what is the primary focus of this study?</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>A) The impact of family interactions on child development.; B) Ways to improve adolescent self-esteem in school settings.; C) How family cohesion and adaptability influence adolescent anxiety symptoms.; D) The benefits of participating in extracurricular activities for mental health.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>This question examines the core research objective outlined in the abstract.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>farmakopoulou2024_greek_anxiety_family_selfesteem.pdf</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>attendance tracking</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>beginner</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
+      <c r="J11" s="4" t="n"/>
+      <c r="K11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>According to the passage, how do social-emotional skills help adolescents in school?</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>A) They improve students' ability to work well with others and manage their own wellbeing.; B) They increase access to extracurricular activities and reduce classroom distractions.; C) They directly boost academic performance through memorization techniques.; D) They provide a clear path for navigating complex social hierarchies within the school.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>The passage states that social-emotional skills help adolescents cope with the demands of school by aiding in positive social interactions and well-being.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>huttunen2025_socioemotional_profiles_anxiety.pdf</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>school social climate</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Which of these is NOT implied as a way for schools to develop protective factors in their pupils?</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>A) Creating a positive school social climate; B) Implementing strict disciplinary policies; C) Fostering strong relationships between staff and students; D) Providing opportunities for student leadership involvement</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>The excerpt focuses on methods to create a supportive environment, which is not the same as strict discipline.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>school social climate</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
+      <c r="J13" s="4" t="n"/>
+      <c r="K13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>According to the passage, which social-emotional skill can help adolescents succeed in school by contributing positively to relationships with others?</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>A) Managing goal- and task-directed behavior; B) Taking care of their own well-being; C) Achieving academic success; D) Establishing and maintaining positive social interactions</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>The passage states that these skills are helpful for adolescents in a school environment, especially when interacting with others.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>huttunen2025_socioemotional_profiles_anxiety.pdf</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>student–teacher relations</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Which of these is MOST directly related to positive student-teacher relationships developing protective factors in pupils according to the excerpt?</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>A) Clear classroom rules and expectations; B) Encouraging extracurricular activities; C) Providing nutritional meals; D) Building a sense of community</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The excerpt highlights the importance of schools in developing protective factors within students. </t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>student–teacher relations</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="4" t="n"/>
+      <c r="K15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Which of the following concepts is MOST closely related to addressing "emotionally based school avoidance"?</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>A) Cognitive restructuring; B) Physical education; C) Standardized testing; D) Extracurricular activities</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>The excerpt focuses on mental wellbeing difficulties as a cause of school non-attendance. Cognitive restructuring is a technique used to address negative thoughts and beliefs.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>cognitive restructuring</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>According to the passage, how does CBT help people manage their feelings or problems?</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>A) By identifying and changing negative thought patterns.; B) By providing emotional support through a listening ear.; C) By prescribing medication to alleviate symptoms.; D) By encouraging individuals to engage in relaxing activities.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The passage states that CBT 'challenges negative thinking and/or behavioral patterns'. </t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>annafreud_seven_ways_support_worried.pdf</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>cognitive restructuring</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="n"/>
+      <c r="I17" s="4" t="n"/>
+      <c r="J17" s="4" t="n"/>
+      <c r="K17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>According to the research excerpt, what is the likelihood of adults who recognize potential Mental Health Problems (MHPs) in children seeking help compared to those who do not?</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>A) Less likely to seek help.; B) More likely to seek help.; C) Equally likely to seek help.; D) The excerpt does not provide information about their likelihood of seeking help.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>The excerpt states that adults who recognize child MHPs are more likely to endorse, seek information on, and access mental health services.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>johnson2023_teacher_mh_literacy_review.pdf</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>parent-teacher collaboration</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="n"/>
+      <c r="K18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>According to the passage, what is an increasing problem in the UK?</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>A) Collaboration between parents and teachers; B) Mental health difficulties among adolescents; C) Diagnosable mental disorders among adults; D) Funding for educational programs</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>The passage highlights the rising prevalence of mental health issues in young people.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>troy2022_school_structural_mh_promotion_review.pdf</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>parent-teacher collaboration</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
+      <c r="J19" s="4" t="n"/>
+      <c r="K19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>According to the paragraph, what is observed regarding the relationship between gender and school bullying (and cyberbullying)?</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>A) Studies show a clear consensus that girls are more likely to be bullied.; B) Some studies suggest that teenage girls are as likely to bully or be bullied as boys.; C) Bullying is mostly perpetrated by boys and cyberbullying is mainly committed by girls.; D) Girls experience more severe forms of bullying than boys.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>The passage states that some studies show teenage girls are as likely to bully or be bullied as boys.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>schlesier2023_bullying_anxiety_absenteeism.pdf</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>graduated exposure</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="n"/>
+      <c r="K20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Which strategy helped the young person transition to full classroom attendance?</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>A) Graded exposure and relaxation strategies; B) Communication sessions with parents; C) Finding a balance between space and support at home; D) Rediscovering her passion for learning</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>The excerpt states that graded exposure, relaxation, and grounding strategies aided the transition.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>graduated exposure</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
+      <c r="J21" s="4" t="n"/>
+      <c r="K21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>According to the excerpt, what can be inferred about the relationship between bullying experiences and school displeasure?</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>A) There is no significant association between bullying experiences and school displeasure.; B) Individuals who experience higher levels of bullying victimization tend to report lower feelings of school displeasure.; C) School displeasure plays a mediating role in the relationship between bullying and absence from school.; D) Individuals who are bullies exhibit less school displeasure compared to those who are victims of bullying.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>The excerpt states that high bullying victimization leads to significantly higher school displeasure.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>schlesier2023_bullying_anxiety_absenteeism.pdf</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>response systems</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
+      <c r="J22" s="4" t="n"/>
+      <c r="K22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>The excerpt suggests that "whole school" approaches to mental health (MH) may have been ineffective partly due to challenges in implementation. What kind of system is being described here?</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>A) Curricula design; B) Feedback and evaluation; C) Resource allocation; D) Teacher training</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>The passage mentions challenges with complex interventions being implemented, implying a need for systems to monitor and adjust.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>troy2022_school_structural_mh_promotion_review.pdf</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>response systems</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="n"/>
+      <c r="I23" s="4" t="n"/>
+      <c r="J23" s="4" t="n"/>
+      <c r="K23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Which of the following statements best reflects the relationship between educational aspirations, school anxiety, and social-emotional skills according to the excerpt?</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>A) Educational aspirations, school anxiety, and social-emotional skills are essentially the same concept.; B) Social-emotional skills influence both educational aspirations and school anxiety but are distinct from them.; C) School anxiety is a result of underdeveloped social-emotional skills.; D) Educational aspirations have no relationship with school anxiety or social-emotional skills.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>The excerpt states that educational aspirations and school anxiety are distinct from social-emotional skills.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>huttunen2025_socioemotional_profiles_anxiety.pdf</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>emotion dysregulation</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="n"/>
+      <c r="J24" s="4" t="n"/>
+      <c r="K24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>According to the passage, which source was used to inform the search strategy for factors related to mental health in schools?</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>A) Environmental factors from a previous review.; B) Clinical guidelines for treating childhood anxiety.; C) Surveys of students' experiences with bullying.; D) Interviews with parents about their children's well-being.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>The passage states that environmental factors from a previous review were used to guide the search strategy.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>troy2022_school_structural_mh_promotion_review.pdf</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>emotion dysregulation</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="n"/>
+      <c r="I25" s="4" t="n"/>
+      <c r="J25" s="4" t="n"/>
+      <c r="K25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>According to the passage, what alternative term is used to describe children who avoid school due to mental health difficulties?</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>A) Comorbid depression; B) Emotionally based school avoidance; C) Academic performance deficit; D) Childhood trauma</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>The passage defines emotionally based school avoidance as a term sometimes used to describe children's non-attendance due to mental health difficulties.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>annafreud_school_attendance_mental_wellbeing.pdf</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>comorbid depression</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="n"/>
+      <c r="I26" s="4" t="n"/>
+      <c r="J26" s="4" t="n"/>
+      <c r="K26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>According to the passage, what is the primary goal of CBT therapy?</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>A) To replace feelings with concrete actions.; B) To provide emotional support and comfort during difficult times.; C) To help individuals modify their thought patterns and behaviors.; D) To encourage patients to rely solely on medication for symptom management.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>The passage states that CBT aims to improve feelings by changing how people think and behave.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>annafreud_seven_ways_support_worried.pdf</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>comorbid depression</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
+      <c r="J27" s="4" t="n"/>
+      <c r="K27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>The excerpt suggests that research into bullying, school anxiety, and school absenteeism is lacking. What implication does this have for understanding the potential internalization of distress among students?</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>A) It makes it difficult to identify which factors contribute most to internalizing symptoms.; B) It confirms that internalizing symptoms are a rare occurrence in school environments.; C) It highlights the importance of studying external behavioral problems instead.; D) It suggests that there is no connection between bullying, anxiety, and absenteeism.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>The lack of research makes it hard to determine the specific influence of these factors on internalizing symptoms.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>schlesier2023_bullying_anxiety_absenteeism.pdf</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>internalizing symptoms</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="4" t="n"/>
+      <c r="K28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>According to the passage, which of the following is a primary reason for focusing on changes within the school environment?</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>A) To understand how internalizing symptoms manifest in different settings.; B) To promote better mental health (MH) by creating a conducive learning environment.; C) To identify specific organizational structures that contribute to stress and anxiety.; D) To encourage physical activity and healthy eating habits among students.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>The passage emphasizes the need to create environments that support better health, including MH.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>troy2022_school_structural_mh_promotion_review.pdf</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>internalizing symptoms</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="4" t="n"/>
+      <c r="J29" s="4" t="n"/>
+      <c r="K29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Which of the following is NOT directly implied as one of the potential consequences junior adolescents might face due to difficulties with academic adaptation?</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>A) Deterioration of health; B) Increased feelings of calmness; C) Behavioral problems; D) Dramatic decrease in academic performance</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>The excerpt discusses negative outcomes related to difficulties adapting to academics.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>shamionov2021_wellbeing_anxiety_variations.pdf</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>autonomic arousal</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="n"/>
+      <c r="J30" s="4" t="n"/>
+      <c r="K30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Which aspect of adolescent well-being does **NOT** feature in this study's goals?</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>A) Family cohesion and adaptability; B) Adolescent anxiety symptoms; C) The impact of peer relationships on mental health; D) Teen self-esteem as a possible mediator</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>The excerpt outlines goals focused on family dynamics and self-esteem's role in anxiety.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>farmakopoulou2024_greek_anxiety_family_selfesteem.pdf</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>autonomic arousal</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="n"/>
+      <c r="J31" s="4" t="n"/>
+      <c r="K31" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>